<commit_message>
feat: Implement Docker support with multi-stage builds, hot reload, and comprehensive documentation
</commit_message>
<xml_diff>
--- a/public/technology_radar_data.xlsx
+++ b/public/technology_radar_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashwath.kumaran\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OrgProjects\technologyRadar\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D95DECF-FA5B-42C5-89A3-E7DCF532E0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E4F08EF-4291-45F2-89EF-96CAD1093291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="66">
   <si>
     <t>Name</t>
   </si>
@@ -213,6 +213,15 @@
   </si>
   <si>
     <t>Evaluate for automation</t>
+  </si>
+  <si>
+    <t>sample</t>
+  </si>
+  <si>
+    <t>Sample</t>
+  </si>
+  <si>
+    <t>Dhanus</t>
   </si>
 </sst>
 </file>
@@ -260,7 +269,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -283,11 +292,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF3D444D"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -296,6 +316,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -752,7 +775,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75C6FFF1-F498-4888-8579-D49426414ACF}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" ht="35.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -855,6 +878,23 @@
       </c>
       <c r="E6" s="2" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="69" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>